<commit_message>
Clean up repo structure: remove stale duplicates, consolidate docs
- Delete extra/ (byte-identical or superseded copies of reports,
  model scores/plots archives, trends, run_frontend.py)
- Delete reports/ (superseded by extra/ copies, now consolidated below)
- Delete root-level loose duplicates: scores_graphs.py,
  Model_Performance_Comparison.png, Frequency Distribution Plots.zip,
  All Model Results.xlsx (kept the newer copy in
  models_scores_and_plots/Models Scores/)
- Delete stray gcm-diagnose.log
- Consolidate reports/, statistical analysis/, and the root user manual
  into docs/

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/models_scores_and_plots/Models Scores/All Model Results.xlsx
+++ b/models_scores_and_plots/Models Scores/All Model Results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research Paper\Solar FYP (Faisal)\Project 1\models_scores_and_plots\Models Scores\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Research Paper\Solar FYP\Project 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7493B8E-1A0F-40B4-942C-8C58A9327D26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6583C1BC-B1A4-488C-851E-623D67132D60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{64B49C39-9350-4B7D-98B6-D002BAE0B7E0}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Model</t>
   </si>
@@ -67,12 +67,6 @@
   </si>
   <si>
     <t>TCN</t>
-  </si>
-  <si>
-    <t>MAE_Train</t>
-  </si>
-  <si>
-    <t>RMSE_Train</t>
   </si>
 </sst>
 </file>
@@ -438,15 +432,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F68D4C-D4DD-4B8B-8EBA-3CD5968F77A8}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="5" width="14.6640625" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,19 +449,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -480,19 +466,13 @@
         <v>0.99329999999999996</v>
       </c>
       <c r="D2" s="2">
-        <v>5.7287999999999997</v>
+        <v>9.6929999999999996</v>
       </c>
       <c r="E2" s="2">
-        <v>9.6929999999999996</v>
-      </c>
-      <c r="F2" s="2">
-        <v>12.0471</v>
-      </c>
-      <c r="G2" s="2">
         <v>22.620699999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -503,108 +483,78 @@
         <v>0.99329999999999996</v>
       </c>
       <c r="D3" s="2">
-        <v>7.3238000000000003</v>
+        <v>9.8764000000000003</v>
       </c>
       <c r="E3" s="2">
-        <v>9.8764000000000003</v>
-      </c>
-      <c r="F3" s="2">
-        <v>16.774999999999999</v>
-      </c>
-      <c r="G3" s="2">
         <v>22.774799999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2">
-        <v>0.98619999999999997</v>
+        <v>0.98760000000000003</v>
       </c>
       <c r="C4" s="2">
-        <v>0.98740000000000006</v>
+        <v>0.98729999999999996</v>
       </c>
       <c r="D4" s="2">
-        <v>17.020600000000002</v>
+        <v>20.186699999999998</v>
       </c>
       <c r="E4" s="2">
-        <v>16.617100000000001</v>
-      </c>
-      <c r="F4" s="2">
-        <v>32.430199999999999</v>
-      </c>
-      <c r="G4" s="2">
-        <v>31.1187</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>31.297699999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="2">
-        <v>0.98680000000000001</v>
+        <v>0.98909999999999998</v>
       </c>
       <c r="C5" s="2">
-        <v>0.9879</v>
+        <v>0.98960000000000004</v>
       </c>
       <c r="D5" s="2">
-        <v>20.5168</v>
+        <v>17.0076</v>
       </c>
       <c r="E5" s="2">
-        <v>19.969899999999999</v>
-      </c>
-      <c r="F5" s="2">
-        <v>31.708200000000001</v>
-      </c>
-      <c r="G5" s="2">
-        <v>30.482700000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>28.219100000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="2">
-        <v>0.99609999999999999</v>
+        <v>0.99590000000000001</v>
       </c>
       <c r="C6" s="2">
-        <v>0.94750000000000001</v>
+        <v>0.94720000000000004</v>
       </c>
       <c r="D6" s="2">
-        <v>8.7817000000000007</v>
+        <v>28.5793</v>
       </c>
       <c r="E6" s="2">
-        <v>27.1432</v>
-      </c>
-      <c r="F6" s="2">
-        <v>17.2011</v>
-      </c>
-      <c r="G6" s="2">
-        <v>63.505499999999998</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>63.694299999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="2">
-        <v>0.99390000000000001</v>
+        <v>0.99360000000000004</v>
       </c>
       <c r="C7" s="2">
-        <v>0.94779999999999998</v>
+        <v>0.94610000000000005</v>
       </c>
       <c r="D7" s="2">
-        <v>11.6608</v>
+        <v>28.827200000000001</v>
       </c>
       <c r="E7" s="2">
-        <v>27.8596</v>
-      </c>
-      <c r="F7" s="2">
-        <v>21.5259</v>
-      </c>
-      <c r="G7" s="2">
-        <v>63.339799999999997</v>
+        <v>64.38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>